<commit_message>
Both datasets successfully run through Script 2. Next up: more in-depth analysis
</commit_message>
<xml_diff>
--- a/Cell data Sara A549/2025_10_30/Multiplicity X-rays 30-10.xlsx
+++ b/Cell data Sara A549/2025_10_30/Multiplicity X-rays 30-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaan\Documents\#Master Degree\Thesis\Thesis_project\Cell data Sara A549\2025_10_30\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772886E5-BABF-4060-8333-B52C42BED726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D623B1F-EFEE-4C42-87DF-4DAC470D452D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -503,9 +503,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
@@ -832,40 +830,42 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1">
+      <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1">
+      <c r="B1">
         <v>2</v>
       </c>
-      <c r="C1" s="1">
+      <c r="C1">
         <v>3</v>
       </c>
-      <c r="D1" s="1">
+      <c r="D1">
         <v>4</v>
       </c>
-      <c r="E1" s="1">
+      <c r="E1">
         <v>5</v>
       </c>
-      <c r="F1" s="1">
+      <c r="F1">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2">
         <v>0.86848635200000002</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>0.10669975199999999</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>1.2406947999999999E-2</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
         <v>9.9255579999999993E-3</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>2.48139E-3</v>
       </c>
     </row>

</xml_diff>